<commit_message>
Platform: saved decisions, two-person approvals, delta loads, personal data, edits, company model, demo hub
- si2_common/store.py + persist.py: SME decisions saved (SQLite or SQL Server) and restored per app
- approvals_ui.py: maker-checker for rating factors, rule sets, NCCI submissions, load plan, migration sign-off
- initial load: PII detection/masking + Data steward role, pick-list code descriptions, bureau-style
  edits with quarantine, type-2 delta loads, hand-off to migration Steps 1-9
- registry.py: company canonical model with where-used across all apps (Canonical app)
- branding: demo hub links and guided tours in every app
- tests/test_platform.py: 12 tests

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Age6rLnmfbYcfSXp1dSyHh
</commit_message>
<xml_diff>
--- a/migrate/initial_load_samples/policy_claims.xlsx
+++ b/migrate/initial_load_samples/policy_claims.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="107">
   <si>
     <t>POL_NO</t>
   </si>
@@ -29,6 +29,12 @@
     <t>INSURED_NM</t>
   </si>
   <si>
+    <t>INSURED_TIN</t>
+  </si>
+  <si>
+    <t>INSURED_EMAIL</t>
+  </si>
+  <si>
     <t>STATE_CD</t>
   </si>
   <si>
@@ -95,6 +101,66 @@
     <t>Priya Patel</t>
   </si>
   <si>
+    <t>900-70-1000</t>
+  </si>
+  <si>
+    <t>901-70-1000</t>
+  </si>
+  <si>
+    <t>910-71-1037</t>
+  </si>
+  <si>
+    <t>920-72-1074</t>
+  </si>
+  <si>
+    <t>921-72-1074</t>
+  </si>
+  <si>
+    <t>930-73-1111</t>
+  </si>
+  <si>
+    <t>940-74-1148</t>
+  </si>
+  <si>
+    <t>941-74-1148</t>
+  </si>
+  <si>
+    <t>950-75-1185</t>
+  </si>
+  <si>
+    <t>960-76-1222</t>
+  </si>
+  <si>
+    <t>961-76-1222</t>
+  </si>
+  <si>
+    <t>970-77-1259</t>
+  </si>
+  <si>
+    <t>maria.lopez@example.com</t>
+  </si>
+  <si>
+    <t>james.carter@example.com</t>
+  </si>
+  <si>
+    <t>ana.silva@example.com</t>
+  </si>
+  <si>
+    <t>robert.king@example.com</t>
+  </si>
+  <si>
+    <t>linda.chen@example.com</t>
+  </si>
+  <si>
+    <t>kevin.brown@example.com</t>
+  </si>
+  <si>
+    <t>acme.delivery@example.com</t>
+  </si>
+  <si>
+    <t>priya.patel@example.com</t>
+  </si>
+  <si>
     <t>FL</t>
   </si>
   <si>
@@ -131,7 +197,7 @@
     <t>30303</t>
   </si>
   <si>
-    <t>43215</t>
+    <t>4321</t>
   </si>
   <si>
     <t>08608</t>
@@ -243,6 +309,9 @@
   </si>
   <si>
     <t>CL-0009</t>
+  </si>
+  <si>
+    <t>CL-0010</t>
   </si>
   <si>
     <t>C</t>
@@ -602,10 +671,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:12">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -636,10 +705,16 @@
       <c r="J1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10">
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B2" s="1">
         <v>45292</v>
@@ -648,30 +723,36 @@
         <v>45658</v>
       </c>
       <c r="D2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F2" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="G2" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="H2" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="I2" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="J2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10">
+        <v>66</v>
+      </c>
+      <c r="K2" t="s">
+        <v>78</v>
+      </c>
+      <c r="L2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B3" s="1">
         <v>45658</v>
@@ -680,30 +761,36 @@
         <v>46023</v>
       </c>
       <c r="D3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E3" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F3" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="G3" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="H3" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="I3" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="J3" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10">
+        <v>67</v>
+      </c>
+      <c r="K3" t="s">
+        <v>78</v>
+      </c>
+      <c r="L3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
       <c r="A4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B4" s="1">
         <v>45323</v>
@@ -712,30 +799,36 @@
         <v>45689</v>
       </c>
       <c r="D4" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E4" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F4" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="G4" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="H4" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="I4" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="J4" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10">
+        <v>68</v>
+      </c>
+      <c r="K4" t="s">
+        <v>79</v>
+      </c>
+      <c r="L4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B5" s="1">
         <v>45352</v>
@@ -744,30 +837,36 @@
         <v>45717</v>
       </c>
       <c r="D5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E5" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F5" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="G5" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="H5" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="I5" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="J5" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10">
+        <v>69</v>
+      </c>
+      <c r="K5" t="s">
+        <v>80</v>
+      </c>
+      <c r="L5" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B6" s="1">
         <v>45717</v>
@@ -776,30 +875,36 @@
         <v>46082</v>
       </c>
       <c r="D6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E6" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="F6" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="G6" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="H6" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="I6" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="J6" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10">
+        <v>70</v>
+      </c>
+      <c r="K6" t="s">
+        <v>80</v>
+      </c>
+      <c r="L6" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B7" s="1">
         <v>45383</v>
@@ -808,30 +913,36 @@
         <v>45748</v>
       </c>
       <c r="D7" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E7" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F7" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="G7" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="H7" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="I7" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="J7" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10">
+        <v>71</v>
+      </c>
+      <c r="K7" t="s">
+        <v>78</v>
+      </c>
+      <c r="L7" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B8" s="1">
         <v>45413</v>
@@ -840,30 +951,36 @@
         <v>45778</v>
       </c>
       <c r="D8" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E8" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F8" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="G8" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="H8" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="I8" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="J8" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10">
+        <v>72</v>
+      </c>
+      <c r="K8" t="s">
+        <v>79</v>
+      </c>
+      <c r="L8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
       <c r="A9" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B9" s="1">
         <v>45778</v>
@@ -872,30 +989,36 @@
         <v>46143</v>
       </c>
       <c r="D9" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E9" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="F9" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="G9" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="H9" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="I9" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="J9" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10">
+        <v>73</v>
+      </c>
+      <c r="K9" t="s">
+        <v>79</v>
+      </c>
+      <c r="L9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
       <c r="A10" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B10" s="1">
         <v>45444</v>
@@ -904,30 +1027,36 @@
         <v>45809</v>
       </c>
       <c r="D10" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E10" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="F10" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="G10" t="s">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="H10" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="I10" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="J10" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10">
+        <v>74</v>
+      </c>
+      <c r="K10" t="s">
+        <v>80</v>
+      </c>
+      <c r="L10" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
       <c r="A11" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B11" s="1">
         <v>45474</v>
@@ -936,30 +1065,36 @@
         <v>45839</v>
       </c>
       <c r="D11" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E11" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="F11" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="G11" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="H11" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="I11" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="J11" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10">
+        <v>75</v>
+      </c>
+      <c r="K11" t="s">
+        <v>78</v>
+      </c>
+      <c r="L11" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
       <c r="A12" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B12" s="1">
         <v>45839</v>
@@ -968,30 +1103,36 @@
         <v>46204</v>
       </c>
       <c r="D12" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E12" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="F12" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="G12" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="H12" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="I12" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="J12" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10">
+        <v>76</v>
+      </c>
+      <c r="K12" t="s">
+        <v>78</v>
+      </c>
+      <c r="L12" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
       <c r="A13" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B13" s="1">
         <v>45505</v>
@@ -1000,25 +1141,31 @@
         <v>45870</v>
       </c>
       <c r="D13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E13" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="F13" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="G13" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="H13" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="I13" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="J13" t="s">
-        <v>60</v>
+        <v>77</v>
+      </c>
+      <c r="K13" t="s">
+        <v>79</v>
+      </c>
+      <c r="L13" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -1028,38 +1175,38 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" t="s">
-        <v>61</v>
+        <v>83</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>62</v>
+        <v>84</v>
       </c>
       <c r="D1" t="s">
-        <v>63</v>
+        <v>85</v>
       </c>
       <c r="E1" t="s">
-        <v>64</v>
+        <v>86</v>
       </c>
       <c r="F1" t="s">
-        <v>65</v>
+        <v>87</v>
       </c>
       <c r="G1" t="s">
-        <v>66</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>67</v>
+        <v>89</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C2" s="1">
         <v>45591</v>
@@ -1068,10 +1215,10 @@
         <v>45594</v>
       </c>
       <c r="E2" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="F2" t="s">
-        <v>79</v>
+        <v>102</v>
       </c>
       <c r="G2">
         <v>8529.379999999999</v>
@@ -1079,10 +1226,10 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>68</v>
+        <v>90</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C3" s="1">
         <v>45871</v>
@@ -1091,10 +1238,10 @@
         <v>45872</v>
       </c>
       <c r="E3" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="F3" t="s">
-        <v>80</v>
+        <v>103</v>
       </c>
       <c r="G3">
         <v>5009.98</v>
@@ -1102,10 +1249,10 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>69</v>
+        <v>91</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C4" s="1">
         <v>45547</v>
@@ -1114,10 +1261,10 @@
         <v>45551</v>
       </c>
       <c r="E4" t="s">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="F4" t="s">
-        <v>79</v>
+        <v>102</v>
       </c>
       <c r="G4">
         <v>2776.34</v>
@@ -1125,10 +1272,10 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>70</v>
+        <v>92</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C5" s="1">
         <v>46024</v>
@@ -1137,10 +1284,10 @@
         <v>46042</v>
       </c>
       <c r="E5" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="F5" t="s">
-        <v>81</v>
+        <v>104</v>
       </c>
       <c r="G5">
         <v>876.88</v>
@@ -1148,10 +1295,10 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>71</v>
+        <v>93</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C6" s="1">
         <v>45739</v>
@@ -1160,10 +1307,10 @@
         <v>45745</v>
       </c>
       <c r="E6" t="s">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="F6" t="s">
-        <v>82</v>
+        <v>105</v>
       </c>
       <c r="G6">
         <v>6995.06</v>
@@ -1171,10 +1318,10 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>72</v>
+        <v>94</v>
       </c>
       <c r="B7" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C7" s="1">
         <v>46020</v>
@@ -1183,10 +1330,10 @@
         <v>46031</v>
       </c>
       <c r="E7" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="F7" t="s">
-        <v>83</v>
+        <v>106</v>
       </c>
       <c r="G7">
         <v>7149.42</v>
@@ -1194,10 +1341,10 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>73</v>
+        <v>95</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C8" s="1">
         <v>45778</v>
@@ -1206,10 +1353,10 @@
         <v>45787</v>
       </c>
       <c r="E8" t="s">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="F8" t="s">
-        <v>81</v>
+        <v>104</v>
       </c>
       <c r="G8">
         <v>6565.01</v>
@@ -1217,10 +1364,10 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>74</v>
+        <v>96</v>
       </c>
       <c r="B9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C9" s="1">
         <v>45886</v>
@@ -1229,10 +1376,10 @@
         <v>45889</v>
       </c>
       <c r="E9" t="s">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="F9" t="s">
-        <v>80</v>
+        <v>103</v>
       </c>
       <c r="G9">
         <v>6814.27</v>
@@ -1240,10 +1387,10 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
-        <v>75</v>
+        <v>97</v>
       </c>
       <c r="B10" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C10" s="1">
         <v>45765</v>
@@ -1252,13 +1399,36 @@
         <v>45778</v>
       </c>
       <c r="E10" t="s">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="F10" t="s">
-        <v>80</v>
+        <v>103</v>
       </c>
       <c r="G10">
         <v>6881.14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" t="s">
+        <v>98</v>
+      </c>
+      <c r="B11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="1">
+        <v>45383</v>
+      </c>
+      <c r="D11" s="1">
+        <v>45378</v>
+      </c>
+      <c r="E11" t="s">
+        <v>100</v>
+      </c>
+      <c r="F11" t="s">
+        <v>103</v>
+      </c>
+      <c r="G11">
+        <v>2500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>